<commit_message>
Restore all files deleted in Task 7 - will review manually before any future deletions
</commit_message>
<xml_diff>
--- a/Castlehold_Final_Palette.xlsx
+++ b/Castlehold_Final_Palette.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nataliebaldacci/Documents/GitHub/DADU-Homebody-Projects/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3979294C-C246-DB47-BE9C-974912138EB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A70D72F7-61BC-504E-9A4C-D595BDD66760}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="53940" yWindow="1580" windowWidth="28320" windowHeight="19860" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="20880" yWindow="680" windowWidth="34560" windowHeight="19820" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Brand Palette" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="269" uniqueCount="158">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="272" uniqueCount="159">
   <si>
     <t>Name</t>
   </si>
@@ -496,13 +496,16 @@
   </si>
   <si>
     <t>https://nataliebaldacci.github.io/DADU-Homebody-Projects/homeowner_portal.html</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#B8AD9A </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="11">
+  <fonts count="12">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -567,8 +570,14 @@
       <name val="Century Schoolbook"/>
       <family val="1"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="27">
+  <fills count="28">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -698,6 +707,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF7A2A1D"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFB8AD9A"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -729,7 +744,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -835,6 +850,7 @@
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="11" fillId="27" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -844,6 +860,7 @@
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
+      <color rgb="FFB8AD9A"/>
       <color rgb="FF4C5C66"/>
     </mruColors>
   </colors>
@@ -1143,7 +1160,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D47"/>
+  <dimension ref="A1:E53"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -1152,7 +1169,7 @@
     <col min="4" max="4" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="28" customHeight="1">
+    <row r="1" spans="1:5" ht="28" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1166,7 +1183,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="28" customHeight="1">
+    <row r="2" spans="1:5" ht="28" customHeight="1">
       <c r="A2" s="2" t="s">
         <v>4</v>
       </c>
@@ -1174,7 +1191,7 @@
       <c r="C2" s="2"/>
       <c r="D2" s="2"/>
     </row>
-    <row r="3" spans="1:4" ht="28" customHeight="1">
+    <row r="3" spans="1:5" ht="28" customHeight="1">
       <c r="A3" s="3" t="s">
         <v>5</v>
       </c>
@@ -1188,7 +1205,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="28" customHeight="1">
+    <row r="4" spans="1:5" ht="28" customHeight="1">
       <c r="A4" s="3" t="s">
         <v>8</v>
       </c>
@@ -1202,7 +1219,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="28" customHeight="1">
+    <row r="5" spans="1:5" ht="28" customHeight="1">
       <c r="A5" s="3" t="s">
         <v>11</v>
       </c>
@@ -1216,7 +1233,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="28" customHeight="1">
+    <row r="6" spans="1:5" ht="28" customHeight="1">
       <c r="A6" s="3" t="s">
         <v>14</v>
       </c>
@@ -1230,7 +1247,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="28" customHeight="1">
+    <row r="7" spans="1:5" ht="28" customHeight="1">
       <c r="A7" s="3" t="s">
         <v>17</v>
       </c>
@@ -1244,7 +1261,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ht="28" customHeight="1">
+    <row r="8" spans="1:5" ht="28" customHeight="1">
       <c r="A8" s="2" t="s">
         <v>20</v>
       </c>
@@ -1252,7 +1269,7 @@
       <c r="C8" s="2"/>
       <c r="D8" s="2"/>
     </row>
-    <row r="9" spans="1:4" ht="28" customHeight="1">
+    <row r="9" spans="1:5" ht="28" customHeight="1">
       <c r="A9" s="3" t="s">
         <v>21</v>
       </c>
@@ -1266,7 +1283,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="10" spans="1:4" ht="28" customHeight="1">
+    <row r="10" spans="1:5" ht="28" customHeight="1">
       <c r="A10" s="3" t="s">
         <v>24</v>
       </c>
@@ -1280,7 +1297,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="11" spans="1:4" ht="28" customHeight="1">
+    <row r="11" spans="1:5" ht="28" customHeight="1">
       <c r="A11" s="3" t="s">
         <v>27</v>
       </c>
@@ -1294,7 +1311,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="12" spans="1:4" ht="28" customHeight="1">
+    <row r="12" spans="1:5" ht="28" customHeight="1">
       <c r="A12" s="3" t="s">
         <v>30</v>
       </c>
@@ -1307,8 +1324,11 @@
       <c r="D12" s="13" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="13" spans="1:4" ht="28" customHeight="1">
+      <c r="E12" s="37" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ht="28" customHeight="1">
       <c r="A13" s="2" t="s">
         <v>33</v>
       </c>
@@ -1316,7 +1336,7 @@
       <c r="C13" s="2"/>
       <c r="D13" s="2"/>
     </row>
-    <row r="14" spans="1:4" ht="28" customHeight="1">
+    <row r="14" spans="1:5" ht="28" customHeight="1">
       <c r="A14" s="3" t="s">
         <v>34</v>
       </c>
@@ -1330,7 +1350,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="15" spans="1:4" ht="28" customHeight="1">
+    <row r="15" spans="1:5" ht="28" customHeight="1">
       <c r="A15" s="2" t="s">
         <v>37</v>
       </c>
@@ -1338,7 +1358,7 @@
       <c r="C15" s="2"/>
       <c r="D15" s="2"/>
     </row>
-    <row r="16" spans="1:4" ht="28" customHeight="1">
+    <row r="16" spans="1:5" ht="28" customHeight="1">
       <c r="A16" s="3" t="s">
         <v>38</v>
       </c>
@@ -1648,8 +1668,17 @@
         <v>35</v>
       </c>
     </row>
+    <row r="53" spans="3:4">
+      <c r="C53" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="D53" s="15" t="s">
+        <v>39</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
 

</xml_diff>